<commit_message>
Add PDF and CSV versions of control tracker for GitHub preview
</commit_message>
<xml_diff>
--- a/docs/05-grc-control-tracker.xlsx
+++ b/docs/05-grc-control-tracker.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Control Tracker'!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Control Tracker'!$A$1:$I$94</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -1330,7 +1331,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1519,7 +1520,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1530,7 +1531,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:I94"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3673,7 +3674,7 @@
   <autoFilter ref="A1:I94"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>